<commit_message>
Update Philly BYOB Restaurant google form_with_websites_20251104_190915_with_emails_20251104_193538.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant google form_with_websites_20251104_190915_with_emails_20251104_193538.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant google form_with_websites_20251104_190915_with_emails_20251104_193538.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CCF1EF-977D-4893-B8CD-BE9B9245B2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C74C90-7D31-4288-811F-3BD624A398D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -829,6 +842,8 @@
   <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="4" max="4" width="27.5" customWidth="1"/>
     <col min="12" max="12" width="22.5" customWidth="1"/>
     <col min="13" max="13" width="26.5" customWidth="1"/>
   </cols>

</xml_diff>